<commit_message>
Stage daily FRA news candidates
</commit_message>
<xml_diff>
--- a/content/news.xlsx
+++ b/content/news.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O309"/>
+  <dimension ref="A1:O310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19429,7 +19429,6 @@
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="D307" t="inlineStr"/>
       <c r="E307" t="inlineStr">
         <is>
           <t>Frankfurt Airport</t>
@@ -19460,8 +19459,6 @@
           <t>review</t>
         </is>
       </c>
-      <c r="K307" t="inlineStr"/>
-      <c r="L307" t="inlineStr"/>
       <c r="M307" t="inlineStr">
         <is>
           <t>review</t>
@@ -19494,7 +19491,6 @@
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="D308" t="inlineStr"/>
       <c r="E308" t="inlineStr">
         <is>
           <t>Frankfurt Airport</t>
@@ -19525,8 +19521,6 @@
           <t>review</t>
         </is>
       </c>
-      <c r="K308" t="inlineStr"/>
-      <c r="L308" t="inlineStr"/>
       <c r="M308" t="inlineStr">
         <is>
           <t>review</t>
@@ -19559,7 +19553,6 @@
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="D309" t="inlineStr"/>
       <c r="E309" t="inlineStr">
         <is>
           <t>Frankfurt Airport</t>
@@ -19590,8 +19583,6 @@
           <t>review</t>
         </is>
       </c>
-      <c r="K309" t="inlineStr"/>
-      <c r="L309" t="inlineStr"/>
       <c r="M309" t="inlineStr">
         <is>
           <t>review</t>
@@ -19603,6 +19594,71 @@
         </is>
       </c>
       <c r="O309" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>auto-845442d2f0b8</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Jericoacoara wird dritter Fraport-Flughafen in Brasilien</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr"/>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Automatisch gefundener Kandidat. Fakten, FRA-Bezug und Quelle vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>FRANKFURT - Fraport expandiert in Südamerika. Der Frankfurter Flughafenbetreiber übernimmt den Betrieb eines dritten Flughafens ins Brasilien - unter dem Dach einer bestehenden Konzession für den Flughafen Fortaleza betreibt Fraport jetzt auch den Airport in Jericoacoara. Die Konzession läuft bis 2047.</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>aero.de</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>https://www.aero.de/news-53542/Jericoacoara-wird-dritter-Fraport-Flughafen-in-Brasilien.html</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="K310" t="inlineStr"/>
+      <c r="L310" t="inlineStr"/>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="N310" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O310" t="inlineStr">
         <is>
           <t>no</t>
         </is>

</xml_diff>